<commit_message>
Actualiza los datos relevados del resto de grupos, actualiza salida en funcion del DATASOURCE
</commit_message>
<xml_diff>
--- a/RESULTADOS.xlsx
+++ b/RESULTADOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTUDIO\Downloads\TP-IO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frsfutneduar-my.sharepoint.com/personal/lzeballos_frsf_utn_edu_ar/Documents/Escritorio/Facultad/io/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1019D43-3347-4AC3-B7A2-FCF292AB6F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESULTADOS ENVIOS (X)" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <definedName name="LECHE_DESCREMADA_ENVIADA_A_SANTA_FE" comment="Resultados del solver para LD. Expresa la cantidad de leche descremada que la planta J envia a la planta de Santa Fe.">'RESULTADOS ENVIOS A SF (LD)'!$C$2:$C$3</definedName>
     <definedName name="LECHE_PROCESADA" comment="Resultados del solver para Y. Expresa la cantidad de leche equivalente que fue procesada en cada planta.">'RESULTADOS PRODUCCION (Y)'!$C$2:$C$4</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -603,14 +603,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D97"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -624,7 +624,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -638,7 +638,7 @@
         <v>546191.91</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
@@ -652,7 +652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -666,7 +666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
@@ -680,7 +680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>3</v>
       </c>
@@ -694,7 +694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
@@ -708,7 +708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>3</v>
       </c>
@@ -722,7 +722,7 @@
         <v>218476.764</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>3</v>
       </c>
@@ -736,7 +736,7 @@
         <v>145651.17600000001</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>3</v>
       </c>
@@ -750,7 +750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>3</v>
       </c>
@@ -764,7 +764,7 @@
         <v>303439.95</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>3</v>
       </c>
@@ -778,7 +778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>3</v>
       </c>
@@ -792,7 +792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
         <v>11</v>
       </c>
@@ -806,7 +806,7 @@
         <v>281371.58999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>11</v>
       </c>
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>11</v>
       </c>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>11</v>
       </c>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>11</v>
       </c>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>11</v>
       </c>
@@ -876,7 +876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>11</v>
       </c>
@@ -890,7 +890,7 @@
         <v>112548.63599999998</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
         <v>11</v>
       </c>
@@ -904,7 +904,7 @@
         <v>75032.423999999985</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>11</v>
       </c>
@@ -918,7 +918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
         <v>11</v>
       </c>
@@ -932,7 +932,7 @@
         <v>156317.54999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
         <v>11</v>
       </c>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>11</v>
       </c>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>12</v>
       </c>
@@ -974,7 +974,7 @@
         <v>39919.5</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>12</v>
       </c>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>12</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>12</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>12</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>12</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>12</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>15967.8</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>12</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>10645.199999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>12</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>12</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>22177.5</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>12</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>12</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>13</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>114608.30437959186</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>13</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>13</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>13</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>13</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>13</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>13</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>5450.0579999999991</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>13</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>3633.3719999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
         <v>13</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>13</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>7569.5249999999996</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>13</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="9" t="s">
         <v>13</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>14</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>96808.5</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>14</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>14</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="7" t="s">
         <v>14</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
         <v>14</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>14</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>14</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>38723.4</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="7" t="s">
         <v>14</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
         <v>14</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="7" t="s">
         <v>14</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>53782.5</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="7" t="s">
         <v>14</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>14</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>25815.599999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>15</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>17995.5</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>15</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>15</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="7" t="s">
         <v>15</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="7" t="s">
         <v>15</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>15</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="7" t="s">
         <v>15</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>15</v>
       </c>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>15</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="7" t="s">
         <v>15</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>9997.5</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="7" t="s">
         <v>15</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>7198.2</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="9" t="s">
         <v>15</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>4798.8</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>16</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>218609.55000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="7" t="s">
         <v>16</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="7" t="s">
         <v>16</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="7" t="s">
         <v>16</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="7" t="s">
         <v>16</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="7" t="s">
         <v>16</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="7" t="s">
         <v>16</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>87443.819999999992</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="7" t="s">
         <v>16</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>58295.88</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="7" t="s">
         <v>16</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="7" t="s">
         <v>16</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>121449.75</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="7" t="s">
         <v>16</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
         <v>16</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>17</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>70333.24500000001</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="7" t="s">
         <v>17</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="7" t="s">
         <v>17</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="7" t="s">
         <v>17</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="7" t="s">
         <v>17</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="7" t="s">
         <v>17</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="7" t="s">
         <v>17</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>28133.297999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="7" t="s">
         <v>17</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>18755.531999999999</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="7" t="s">
         <v>17</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="7" t="s">
         <v>17</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>39074.025000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="7" t="s">
         <v>17</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="9" t="s">
         <v>17</v>
       </c>
@@ -1976,12 +1976,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05649807-5BCA-4CDC-892B-C264250D9331}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>4480622.5343550006</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>2262609.3395699998</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2033,14 +2033,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85634DFB-2640-45DB-972B-03B088998E42}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2062,7 +2062,7 @@
         <v>89559.050968955693</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>

</xml_diff>